<commit_message>
FIX: repair 2. data cause lack of logic in code
</commit_message>
<xml_diff>
--- a/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
+++ b/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tanda\Desktop\NCKH\TSF_Github\Drafts\Temp Prediction\models\checkpoints\ML\Random Forest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14498D36-20E9-4C26-985F-BBEFD02999C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB8B756-45A4-4C5A-8264-3040E8479025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2928" yWindow="1968" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
   <si>
     <t>step_size = 15</t>
   </si>
@@ -79,6 +79,30 @@
   </si>
   <si>
     <t>max_depth_29</t>
+  </si>
+  <si>
+    <t>Lagging feature</t>
+  </si>
+  <si>
+    <t>max_features_None</t>
+  </si>
+  <si>
+    <t>4th</t>
+  </si>
+  <si>
+    <t>n_estimators_421</t>
+  </si>
+  <si>
+    <t>local</t>
+  </si>
+  <si>
+    <t>max_depth_43</t>
+  </si>
+  <si>
+    <t>max_features_sqrt</t>
+  </si>
+  <si>
+    <t>max_depth_36</t>
   </si>
 </sst>
 </file>
@@ -121,7 +145,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -136,19 +160,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -183,26 +194,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,71 +493,79 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" customWidth="1"/>
     <col min="15" max="15" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>1</v>
       </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4"/>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="2" t="s">
+      <c r="I3" s="4"/>
+      <c r="J3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="4"/>
-      <c r="M3" s="5" t="s">
+      <c r="M3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="P3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="S3" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="9"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="5">
+        <v>0.90822991905697503</v>
+      </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="10">
+      <c r="G4" s="7">
         <v>0.80939190320593102</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="8">
+      <c r="J4" s="6">
         <v>0.84004313076820802</v>
       </c>
       <c r="K4" s="1"/>
@@ -555,109 +573,209 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="8">
+      <c r="P4" s="6">
         <v>0.881730360867092</v>
       </c>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="8" t="s">
+      <c r="C5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="5">
+        <v>0.885687182873382</v>
+      </c>
+      <c r="E5" s="8">
+        <v>2.4799999999999999E-2</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="7">
         <v>0.80613165498637895</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="8">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="8">
+      <c r="J5" s="6">
         <v>0.82469552004505597</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="8">
         <v>1.83E-2</v>
       </c>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="5">
+        <v>0.79420416883792899</v>
+      </c>
       <c r="N5" s="1"/>
-      <c r="O5" s="8" t="s">
+      <c r="O5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="P5" s="8">
+      <c r="P5" s="6">
         <v>0.86712953924796599</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="Q5" s="8">
         <v>1.66E-2</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="8" t="s">
+      <c r="C6" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="5">
+        <v>0.87309994935092194</v>
+      </c>
+      <c r="E6" s="8">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="6">
         <v>0.80343492090786095</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="8">
         <v>3.3E-3</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="6">
         <v>0.82464333239207999</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="8">
         <v>1E-4</v>
       </c>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="8" t="s">
+      <c r="L6" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="5">
+        <v>0.78548993139516299</v>
+      </c>
+      <c r="N6" s="8">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="Q6" s="1"/>
+      <c r="P6" s="6">
+        <v>0.86684898064386695</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>2.9999999999999997E-4</v>
+      </c>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
+      <c r="C7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="5">
+        <v>0.87307721886435297</v>
+      </c>
+      <c r="E7" s="9">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="6">
+        <v>0.80343492090786095</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="6">
+        <v>0.82464333239207999</v>
+      </c>
+      <c r="K7" s="9">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" s="5">
+        <v>0.78548993139516299</v>
+      </c>
+      <c r="N7" s="9">
+        <v>0</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="P7" s="6">
+        <v>0.86684898064386695</v>
+      </c>
+      <c r="Q7" s="9">
+        <v>0</v>
+      </c>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0.87307721886435197</v>
+      </c>
+      <c r="E8" s="9">
+        <v>0</v>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="5">
+        <v>0.82464333239207899</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="5">
+        <v>0.78548993139516299</v>
+      </c>
+      <c r="N8" s="9">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
ADD: add 5.4 1.eda code
</commit_message>
<xml_diff>
--- a/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
+++ b/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tanda\Desktop\NCKH\TSF_Github\Drafts\Temp Prediction\models\checkpoints\ML\Random Forest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB8B756-45A4-4C5A-8264-3040E8479025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23A6896-27BE-4202-B7D7-6B935A2EDD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2928" yWindow="1968" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>step_size = 15</t>
   </si>
@@ -66,50 +66,44 @@
     <t>Default</t>
   </si>
   <si>
-    <t>n_estimators_807</t>
-  </si>
-  <si>
-    <t>max_depth_22</t>
-  </si>
-  <si>
-    <t>n_estimators_871</t>
-  </si>
-  <si>
     <t>n_estimators_1000</t>
   </si>
   <si>
-    <t>max_depth_29</t>
-  </si>
-  <si>
     <t>Lagging feature</t>
   </si>
   <si>
-    <t>max_features_None</t>
-  </si>
-  <si>
     <t>4th</t>
   </si>
   <si>
-    <t>n_estimators_421</t>
-  </si>
-  <si>
     <t>local</t>
   </si>
   <si>
-    <t>max_depth_43</t>
-  </si>
-  <si>
     <t>max_features_sqrt</t>
   </si>
   <si>
-    <t>max_depth_36</t>
+    <t>n_estimators_164</t>
+  </si>
+  <si>
+    <t>n_estimators_935</t>
+  </si>
+  <si>
+    <t>max_depth_861</t>
+  </si>
+  <si>
+    <t>criterion_friedman_mse</t>
+  </si>
+  <si>
+    <t>max_depth_6023</t>
+  </si>
+  <si>
+    <t>min_samples_leaf_1e-05</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -128,13 +122,6 @@
       <color rgb="FFCCCCCC"/>
       <name val="Consolas"/>
       <family val="3"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFCCCCCC"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -206,13 +193,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,11 +485,11 @@
   <cols>
     <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" customWidth="1"/>
     <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.33203125" customWidth="1"/>
@@ -520,10 +507,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
@@ -533,7 +520,7 @@
       <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="9" t="s">
         <v>3</v>
       </c>
       <c r="I3" s="4"/>
@@ -556,26 +543,24 @@
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="5">
-        <v>0.90822991905697503</v>
+        <v>0.90822991905697403</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="7">
-        <v>0.80939190320593102</v>
-      </c>
-      <c r="H4" s="1"/>
+      <c r="G4" s="5">
+        <v>0.79617317449543601</v>
+      </c>
+      <c r="H4" s="7"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="6">
-        <v>0.84004313076820802</v>
+      <c r="J4" s="5">
+        <v>0.830333530300705</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
+      <c r="M4" s="6"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
-      <c r="P4" s="6">
-        <v>0.881730360867092</v>
-      </c>
+      <c r="P4" s="6"/>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
@@ -586,46 +571,38 @@
         <v>8</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D5" s="5">
         <v>0.885687182873382</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="11">
         <v>2.4799999999999999E-2</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="7">
-        <v>0.80613165498637895</v>
-      </c>
-      <c r="H5" s="8">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0.82469552004505597</v>
-      </c>
-      <c r="K5" s="8">
-        <v>1.83E-2</v>
-      </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="5">
-        <v>0.79420416883792899</v>
-      </c>
-      <c r="N5" s="1"/>
-      <c r="O5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6">
-        <v>0.86712953924796599</v>
-      </c>
-      <c r="Q5" s="8">
-        <v>1.66E-2</v>
-      </c>
+      <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5">
+        <v>0.79589636114573803</v>
+      </c>
+      <c r="H5" s="7">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="5">
+        <v>0.81353010237009404</v>
+      </c>
+      <c r="K5" s="7">
+        <v>2.0199999999999999E-2</v>
+      </c>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="7"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
@@ -635,50 +612,38 @@
         <v>9</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6" s="5">
         <v>0.87309994935092194</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <v>1.4200000000000001E-2</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0.80343492090786095</v>
+      <c r="F6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="5">
+        <v>0.79589636114573703</v>
       </c>
       <c r="H6" s="8">
-        <v>3.3E-3</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="6">
-        <v>0.82464333239207999</v>
-      </c>
-      <c r="K6" s="8">
-        <v>1E-4</v>
-      </c>
-      <c r="L6" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M6" s="5">
-        <v>0.78548993139516299</v>
-      </c>
-      <c r="N6" s="8">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="P6" s="6">
-        <v>0.86684898064386695</v>
-      </c>
-      <c r="Q6" s="8">
+      <c r="J6" s="5">
+        <v>0.81330649396282595</v>
+      </c>
+      <c r="K6" s="7">
         <v>2.9999999999999997E-4</v>
       </c>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="7"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
@@ -688,88 +653,64 @@
         <v>10</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D7" s="5">
-        <v>0.87307721886435297</v>
-      </c>
-      <c r="E7" s="9">
+        <v>0.87309994935092095</v>
+      </c>
+      <c r="E7" s="8">
         <v>0</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="6">
-        <v>0.80343492090786095</v>
-      </c>
-      <c r="H7" s="9">
+      <c r="F7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="5">
+        <v>0.79589636114573803</v>
+      </c>
+      <c r="H7" s="8">
         <v>0</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0.82464333239207999</v>
-      </c>
-      <c r="K7" s="9">
+      <c r="I7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="5">
+        <v>0.81330649396282595</v>
+      </c>
+      <c r="K7" s="8">
         <v>0</v>
       </c>
-      <c r="L7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="5">
-        <v>0.78548993139516299</v>
-      </c>
-      <c r="N7" s="9">
-        <v>0</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="P7" s="6">
-        <v>0.86684898064386695</v>
-      </c>
-      <c r="Q7" s="9">
-        <v>0</v>
-      </c>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="8"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0.87307721886435197</v>
-      </c>
-      <c r="E8" s="9">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1"/>
+        <v>15</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="6"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J8" s="5">
-        <v>0.82464333239207899</v>
-      </c>
-      <c r="K8" s="9">
+        <v>0.81330649396282595</v>
+      </c>
+      <c r="K8" s="8">
         <v>0</v>
       </c>
-      <c r="L8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="M8" s="5">
-        <v>0.78548993139516299</v>
-      </c>
-      <c r="N8" s="9">
-        <v>0</v>
-      </c>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="8"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>

</xml_diff>

<commit_message>
ADD: sửa lỗi data bị trùng (TSN)
</commit_message>
<xml_diff>
--- a/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
+++ b/Drafts/Temp Prediction/models/checkpoints/ML/Random Forest/RF_Tuning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NCKH\TSF_Github\Drafts\Temp Prediction\models\checkpoints\ML\Random Forest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751B870D-E080-421A-B8C7-C8C5AC0F9570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD2E043-2E1A-4753-96A3-6B5F63DA793B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2928" yWindow="1968" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>step_size = 15</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t>Improve</t>
+  </si>
+  <si>
+    <t>n_estimators_871</t>
+  </si>
+  <si>
+    <t>Valid</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
@@ -596,9 +605,13 @@
       <c r="C3" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="23"/>
+      <c r="D3" s="23" t="s">
+        <v>13</v>
+      </c>
       <c r="E3" s="11"/>
-      <c r="F3" s="12"/>
+      <c r="F3" s="12" t="s">
+        <v>14</v>
+      </c>
       <c r="G3" s="13"/>
       <c r="H3" s="11"/>
       <c r="I3" s="14"/>
@@ -620,7 +633,7 @@
       </c>
       <c r="C4" s="24"/>
       <c r="D4" s="29">
-        <v>0.81988544606893798</v>
+        <v>0.66428535959666402</v>
       </c>
       <c r="E4" s="17"/>
       <c r="F4" s="14"/>
@@ -643,12 +656,14 @@
       <c r="B5" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="26"/>
+      <c r="C5" s="29" t="s">
+        <v>12</v>
+      </c>
       <c r="D5" s="29">
-        <v>0.81106181222210905</v>
+        <v>0.65857322072256996</v>
       </c>
       <c r="E5" s="9">
-        <v>1.0800000000000001E-2</v>
+        <v>8.6E-3</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="7"/>

</xml_diff>